<commit_message>
update short workshop files to 3.9.0
</commit_message>
<xml_diff>
--- a/OS_exercises/openstudio-short/building_data.xlsx
+++ b/OS_exercises/openstudio-short/building_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vuonge\Documents\Reference\OpenStudio_workshop\git\os_workshop\OS_exercises\openstudio-short\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2D3D65E-FD2A-4BA5-A7A0-E8518E812510}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B53ADFC-B3A8-4C3F-825B-F1DF5DCD0B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BE" sheetId="1" r:id="rId1"/>
@@ -32,6 +32,9 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -427,8 +430,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.000000000"/>
+  <numFmts count="1">
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
@@ -770,7 +772,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
@@ -780,9 +782,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -800,7 +799,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -895,75 +893,81 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="46" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1246,18 +1250,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A3:I37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="43.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="29.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="43.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>10</v>
       </c>
@@ -1277,7 +1281,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -1294,7 +1298,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>1</v>
       </c>
@@ -1311,7 +1315,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>2</v>
       </c>
@@ -1328,7 +1332,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>3</v>
       </c>
@@ -1345,7 +1349,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>4</v>
       </c>
@@ -1362,7 +1366,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>5</v>
       </c>
@@ -1379,7 +1383,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>26</v>
       </c>
@@ -1396,7 +1400,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>6</v>
       </c>
@@ -1413,7 +1417,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>25</v>
       </c>
@@ -1424,7 +1428,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>24</v>
       </c>
@@ -1435,7 +1439,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>27</v>
       </c>
@@ -1452,7 +1456,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>40</v>
       </c>
@@ -1469,7 +1473,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>41</v>
       </c>
@@ -1486,7 +1490,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>42</v>
       </c>
@@ -1500,54 +1504,54 @@
         <v>1630</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A19" s="56" t="s">
+    <row r="19" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="56"/>
-      <c r="C19" s="56"/>
-      <c r="D19" s="56"/>
-      <c r="E19" s="56"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="56"/>
-      <c r="H19" s="56"/>
-      <c r="I19" s="56"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B19" s="55"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="55"/>
+      <c r="E19" s="55"/>
+      <c r="F19" s="55"/>
+      <c r="G19" s="55"/>
+      <c r="H19" s="55"/>
+      <c r="I19" s="55"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="D20" t="str">
+      <c r="D20" s="11" t="str">
         <f>C3</f>
         <v>Thermal conductivity [W/(m.K)]</v>
       </c>
-      <c r="E20" t="str">
+      <c r="E20" s="11" t="str">
         <f>D3</f>
         <v>Density [kg/m3]</v>
       </c>
-      <c r="F20" t="str">
+      <c r="F20" s="11" t="str">
         <f>E3</f>
         <v>Specific heat [J/kg.K)]</v>
       </c>
-      <c r="G20" t="str">
+      <c r="G20" s="11" t="str">
         <f>F3</f>
         <v>RSI = L/k [m2K/W]</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="12" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="61" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="56" t="s">
         <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1569,21 +1573,21 @@
         <f>E10</f>
         <v>1000</v>
       </c>
-      <c r="G21" s="9">
+      <c r="G21" s="77">
         <f>C21/D21</f>
         <v>0.11</v>
       </c>
-      <c r="H21" s="64">
+      <c r="H21" s="59">
         <f>SUM(G21:G24)</f>
         <v>5.3398742138364774</v>
       </c>
-      <c r="I21" s="64">
+      <c r="I21" s="59">
         <f>1/H21</f>
         <v>0.18727032884198627</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="62"/>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="58"/>
       <c r="B22" s="2" t="s">
         <v>14</v>
       </c>
@@ -1599,15 +1603,15 @@
       <c r="F22" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G22" s="10">
+      <c r="G22" s="78">
         <f>F12</f>
         <v>0.15</v>
       </c>
-      <c r="H22" s="64"/>
-      <c r="I22" s="64"/>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="62"/>
+      <c r="H22" s="59"/>
+      <c r="I22" s="59"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="58"/>
       <c r="B23" s="2" t="s">
         <v>15</v>
       </c>
@@ -1626,15 +1630,15 @@
         <f t="shared" si="0"/>
         <v>960</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="78">
         <f t="shared" ref="G23:G24" si="1">C23/D23</f>
         <v>5</v>
       </c>
-      <c r="H23" s="64"/>
-      <c r="I23" s="64"/>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="62"/>
+      <c r="H23" s="59"/>
+      <c r="I23" s="59"/>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="58"/>
       <c r="B24" s="2" t="s">
         <v>16</v>
       </c>
@@ -1653,15 +1657,15 @@
         <f t="shared" si="0"/>
         <v>1090</v>
       </c>
-      <c r="G24" s="10">
+      <c r="G24" s="78">
         <f t="shared" si="1"/>
         <v>7.9874213836477984E-2</v>
       </c>
-      <c r="H24" s="64"/>
-      <c r="I24" s="64"/>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="61" t="s">
+      <c r="H24" s="59"/>
+      <c r="I24" s="59"/>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="56" t="s">
         <v>34</v>
       </c>
       <c r="B25" s="1" t="str">
@@ -1684,21 +1688,21 @@
         <f t="shared" si="2"/>
         <v>1090</v>
       </c>
-      <c r="G25" s="9">
+      <c r="G25" s="77">
         <f t="shared" ref="G25:G27" si="3">C25/D25</f>
         <v>7.9874213836477984E-2</v>
       </c>
-      <c r="H25" s="64">
+      <c r="H25" s="59">
         <f>SUM(G25:G27)</f>
         <v>9.3997484276729555</v>
       </c>
-      <c r="I25" s="64">
+      <c r="I25" s="59">
         <f>1/H25</f>
         <v>0.10638582592870142</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A26" s="62"/>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="58"/>
       <c r="B26" s="2" t="s">
         <v>35</v>
       </c>
@@ -1717,15 +1721,15 @@
         <f t="shared" si="4"/>
         <v>960</v>
       </c>
-      <c r="G26" s="10">
+      <c r="G26" s="78">
         <f t="shared" si="3"/>
         <v>9.24</v>
       </c>
-      <c r="H26" s="64"/>
-      <c r="I26" s="64"/>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A27" s="63"/>
+      <c r="H26" s="59"/>
+      <c r="I26" s="59"/>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="57"/>
       <c r="B27" s="3" t="s">
         <v>33</v>
       </c>
@@ -1744,15 +1748,15 @@
         <f t="shared" si="4"/>
         <v>1090</v>
       </c>
-      <c r="G27" s="11">
+      <c r="G27" s="79">
         <f t="shared" si="3"/>
         <v>7.9874213836477984E-2</v>
       </c>
-      <c r="H27" s="64"/>
-      <c r="I27" s="64"/>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A28" s="61" t="s">
+      <c r="H27" s="59"/>
+      <c r="I27" s="59"/>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" s="56" t="s">
         <v>38</v>
       </c>
       <c r="B28" s="5" t="s">
@@ -1773,25 +1777,25 @@
         <f>E10</f>
         <v>1000</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="80">
         <f t="shared" ref="G28:G33" si="5">C28/D28</f>
         <v>0.11</v>
       </c>
-      <c r="H28" s="57">
+      <c r="H28" s="60">
         <f>SUM(G28:G29)</f>
         <v>0.22043478260869565</v>
       </c>
-      <c r="I28" s="59">
+      <c r="I28" s="62">
         <f>1/H28</f>
         <v>4.5364891518737673</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="63"/>
-      <c r="B29" s="12" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" s="57"/>
+      <c r="B29" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C29" s="9">
         <v>1.2699999999999999E-2</v>
       </c>
       <c r="D29" s="3">
@@ -1806,15 +1810,15 @@
         <f t="shared" si="6"/>
         <v>121</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="81">
         <f t="shared" si="5"/>
         <v>0.11043478260869564</v>
       </c>
-      <c r="H29" s="58"/>
-      <c r="I29" s="60"/>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="62" t="s">
+      <c r="H29" s="61"/>
+      <c r="I29" s="63"/>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" s="58" t="s">
         <v>32</v>
       </c>
       <c r="B30" t="s">
@@ -1835,21 +1839,21 @@
         <f t="shared" si="6"/>
         <v>900</v>
       </c>
-      <c r="G30" s="21">
+      <c r="G30" s="82">
         <f t="shared" si="5"/>
         <v>5.1282051282051287E-2</v>
       </c>
-      <c r="H30" s="64">
+      <c r="H30" s="59">
         <f>SUM(G30:G33)</f>
         <v>3.1337200897885933</v>
       </c>
-      <c r="I30" s="64">
+      <c r="I30" s="59">
         <f>1/H30</f>
         <v>0.31910954754975002</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="62"/>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" s="58"/>
       <c r="B31" t="s">
         <v>31</v>
       </c>
@@ -1868,15 +1872,15 @@
         <f t="shared" si="7"/>
         <v>1500</v>
       </c>
-      <c r="G31" s="21">
+      <c r="G31" s="82">
         <f t="shared" si="5"/>
         <v>1.7857142857142858</v>
       </c>
-      <c r="H31" s="64"/>
-      <c r="I31" s="64"/>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="62"/>
+      <c r="H31" s="59"/>
+      <c r="I31" s="59"/>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="58"/>
       <c r="B32" t="s">
         <v>30</v>
       </c>
@@ -1895,15 +1899,15 @@
         <f t="shared" si="7"/>
         <v>1880</v>
       </c>
-      <c r="G32" s="21">
+      <c r="G32" s="82">
         <f t="shared" si="5"/>
         <v>1.1764705882352942</v>
       </c>
-      <c r="H32" s="64"/>
-      <c r="I32" s="64"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="62"/>
+      <c r="H32" s="59"/>
+      <c r="I32" s="59"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="58"/>
       <c r="B33" t="s">
         <v>28</v>
       </c>
@@ -1922,54 +1926,49 @@
         <f>E14</f>
         <v>1630</v>
       </c>
-      <c r="G33" s="21">
+      <c r="G33" s="82">
         <f t="shared" si="5"/>
         <v>0.12025316455696203</v>
       </c>
-      <c r="H33" s="64"/>
-      <c r="I33" s="64"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="20" t="s">
+      <c r="H33" s="59"/>
+      <c r="I33" s="59"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="15">
+      <c r="B34" s="11"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="13"/>
+      <c r="I34" s="12">
         <v>0.83</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:9" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A36" s="56" t="s">
+    <row r="35" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="1:9" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A36" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="B36" s="56"/>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="56"/>
-      <c r="I36" s="56"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B36" s="55"/>
+      <c r="C36" s="55"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="55"/>
+      <c r="H36" s="55"/>
+      <c r="I36" s="55"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="I30:I33"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="H28:H29"/>
     <mergeCell ref="I28:I29"/>
@@ -1979,6 +1978,11 @@
     <mergeCell ref="I21:I24"/>
     <mergeCell ref="H25:H27"/>
     <mergeCell ref="I25:I27"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="I30:I33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1988,32 +1992,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABD82822-F742-4C76-96A1-B0967C95B862}">
   <dimension ref="A1:G37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="47.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="47.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
         <v>48</v>
       </c>
@@ -2026,11 +2030,11 @@
       <c r="D2" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="19" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>53</v>
       </c>
@@ -2043,11 +2047,11 @@
       <c r="D3" s="2">
         <v>0.2</v>
       </c>
-      <c r="E3" s="24">
+      <c r="E3" s="20">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>54</v>
       </c>
@@ -2060,544 +2064,544 @@
       <c r="D4" s="3">
         <v>0.2</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="21">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="66" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="65" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="67"/>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="68"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="B7" s="66"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="66"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="66"/>
+      <c r="G7" s="67"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="12" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="29">
+      <c r="B9" s="25">
         <v>288</v>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="25">
         <v>0.1</v>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="25">
         <v>0.46</v>
       </c>
-      <c r="E9" s="29">
+      <c r="E9" s="25">
         <v>0</v>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="25">
         <f t="shared" ref="F9:F12" si="0">1-SUM(C9:E9)</f>
         <v>0.43999999999999995</v>
       </c>
-      <c r="G9" s="23"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="18" t="s">
+      <c r="G9" s="19"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="35">
+      <c r="B10" s="31">
         <v>570</v>
       </c>
-      <c r="C10" s="35">
+      <c r="C10" s="31">
         <v>0</v>
       </c>
-      <c r="D10" s="35">
+      <c r="D10" s="31">
         <v>0.3</v>
       </c>
-      <c r="E10" s="35">
+      <c r="E10" s="31">
         <v>0</v>
       </c>
-      <c r="F10" s="35">
+      <c r="F10" s="31">
         <f t="shared" si="0"/>
         <v>0.7</v>
       </c>
-      <c r="G10" s="24"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="G10" s="20"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="35">
+      <c r="B11" s="31">
         <v>1000</v>
       </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35">
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G11" s="20" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="26">
+      <c r="B12" s="22">
         <f>388.8*0.25</f>
         <v>97.2</v>
       </c>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26">
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G12" s="36" t="s">
+      <c r="G12" s="32" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="72" t="s">
+    <row r="14" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="71" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="74"/>
-    </row>
-    <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="37" t="s">
+      <c r="B15" s="72"/>
+      <c r="C15" s="72"/>
+      <c r="D15" s="72"/>
+      <c r="E15" s="72"/>
+      <c r="F15" s="73"/>
+    </row>
+    <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="38" t="s">
+      <c r="C16" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="D16" s="38" t="s">
+      <c r="D16" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="38" t="s">
+      <c r="E16" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="39" t="s">
+      <c r="F16" s="35" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="72" t="s">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" s="71" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="73">
+      <c r="B17" s="72">
         <v>105</v>
       </c>
-      <c r="C17" s="40">
+      <c r="C17" s="36">
         <v>105</v>
       </c>
-      <c r="D17" s="41">
+      <c r="D17" s="37">
         <v>0.29166666666666669</v>
       </c>
-      <c r="E17" s="41">
+      <c r="E17" s="37">
         <v>0.33333333333333331</v>
       </c>
-      <c r="F17" s="51">
+      <c r="F17" s="47">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="75"/>
-      <c r="B18" s="76"/>
-      <c r="C18" s="42">
+    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="74"/>
+      <c r="B18" s="75"/>
+      <c r="C18" s="38">
         <v>105</v>
       </c>
-      <c r="D18" s="43">
+      <c r="D18" s="39">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E18" s="43">
+      <c r="E18" s="39">
         <v>0.95833333333333337</v>
       </c>
-      <c r="F18" s="52">
+      <c r="F18" s="48">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="77" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" s="76" t="s">
         <v>84</v>
       </c>
-      <c r="B19" s="73">
+      <c r="B19" s="72">
         <v>105</v>
       </c>
-      <c r="C19" s="44">
+      <c r="C19" s="40">
         <v>105</v>
       </c>
-      <c r="D19" s="45">
+      <c r="D19" s="41">
         <v>0.29166666666666669</v>
       </c>
-      <c r="E19" s="45">
+      <c r="E19" s="41">
         <v>0.33333333333333331</v>
       </c>
-      <c r="F19" s="53">
+      <c r="F19" s="49">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="77"/>
-      <c r="B20" s="76"/>
-      <c r="C20" s="44">
+    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="76"/>
+      <c r="B20" s="75"/>
+      <c r="C20" s="40">
         <v>70</v>
       </c>
-      <c r="D20" s="45">
+      <c r="D20" s="41">
         <v>0.75</v>
       </c>
-      <c r="E20" s="46">
+      <c r="E20" s="42">
         <v>0.95833333333333337</v>
       </c>
-      <c r="F20" s="54">
+      <c r="F20" s="50">
         <f>70/105</f>
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="72" t="s">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" s="71" t="s">
         <v>85</v>
       </c>
-      <c r="B21" s="73">
+      <c r="B21" s="72">
         <v>570</v>
       </c>
-      <c r="C21" s="40">
+      <c r="C21" s="36">
         <v>570</v>
       </c>
-      <c r="D21" s="41">
+      <c r="D21" s="37">
         <v>0.29166666666666669</v>
       </c>
-      <c r="E21" s="41">
+      <c r="E21" s="37">
         <v>0.2986111111111111</v>
       </c>
-      <c r="F21" s="51">
+      <c r="F21" s="47">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="75"/>
-      <c r="B22" s="76"/>
-      <c r="C22" s="42">
+    <row r="22" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="74"/>
+      <c r="B22" s="75"/>
+      <c r="C22" s="38">
         <v>570</v>
       </c>
-      <c r="D22" s="43">
+      <c r="D22" s="39">
         <v>0.72916666666666663</v>
       </c>
-      <c r="E22" s="43">
+      <c r="E22" s="39">
         <v>0.73958333333333337</v>
       </c>
-      <c r="F22" s="52">
+      <c r="F22" s="48">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="77" t="s">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" s="76" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="73">
+      <c r="B23" s="72">
         <v>1000</v>
       </c>
-      <c r="C23" s="44">
+      <c r="C23" s="40">
         <f>0.95*1000</f>
         <v>950</v>
       </c>
-      <c r="D23" s="45">
+      <c r="D23" s="41">
         <v>0.3125</v>
       </c>
-      <c r="E23" s="45">
+      <c r="E23" s="41">
         <v>0.32291666666666669</v>
       </c>
-      <c r="F23" s="53">
+      <c r="F23" s="49">
         <v>0.95</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="77"/>
-      <c r="B24" s="76"/>
-      <c r="C24" s="44">
+    <row r="24" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="76"/>
+      <c r="B24" s="75"/>
+      <c r="C24" s="40">
         <f>0.95*1000</f>
         <v>950</v>
       </c>
-      <c r="D24" s="45">
+      <c r="D24" s="41">
         <v>0.72916666666666663</v>
       </c>
-      <c r="E24" s="45">
+      <c r="E24" s="41">
         <v>0.73958333333333337</v>
       </c>
-      <c r="F24" s="53">
+      <c r="F24" s="49">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="37" t="s">
+    <row r="25" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="B25" s="38">
+      <c r="B25" s="34">
         <v>288</v>
       </c>
-      <c r="C25" s="38">
+      <c r="C25" s="34">
         <v>288</v>
       </c>
-      <c r="D25" s="47">
+      <c r="D25" s="43">
         <v>0.75</v>
       </c>
-      <c r="E25" s="47">
+      <c r="E25" s="43">
         <v>0.83333333333333337</v>
       </c>
-      <c r="F25" s="55">
+      <c r="F25" s="51">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="48" t="s">
+    <row r="26" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="44" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="42"/>
-      <c r="D26" s="42" t="s">
+      <c r="C26" s="38"/>
+      <c r="D26" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="E26" s="42"/>
-      <c r="F26" s="52">
+      <c r="E26" s="38"/>
+      <c r="F26" s="48">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="49"/>
-      <c r="B27" s="49"/>
-      <c r="C27" s="49"/>
-      <c r="D27" s="49"/>
-      <c r="E27" s="49"/>
-      <c r="F27" s="50"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="49"/>
-      <c r="B28" s="49"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="49"/>
-      <c r="E28" s="49"/>
-      <c r="F28" s="50"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="66" t="s">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" s="45"/>
+      <c r="B27" s="45"/>
+      <c r="C27" s="45"/>
+      <c r="D27" s="45"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="46"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" s="45"/>
+      <c r="B28" s="45"/>
+      <c r="C28" s="45"/>
+      <c r="D28" s="45"/>
+      <c r="E28" s="45"/>
+      <c r="F28" s="46"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="65" t="s">
         <v>67</v>
       </c>
-      <c r="B29" s="67"/>
-      <c r="C29" s="67"/>
-      <c r="D29" s="67"/>
-      <c r="E29" s="67"/>
-      <c r="F29" s="67"/>
-      <c r="G29" s="68"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
+      <c r="B29" s="66"/>
+      <c r="C29" s="66"/>
+      <c r="D29" s="66"/>
+      <c r="E29" s="66"/>
+      <c r="F29" s="66"/>
+      <c r="G29" s="67"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B30" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C30" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="D30" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="E30" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F30" s="15" t="s">
+      <c r="F30" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="G30" s="15" t="s">
+      <c r="G30" s="12" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="18" t="s">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="22">
+      <c r="B31" s="18">
         <v>4</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="C31" s="18" t="s">
         <v>73</v>
       </c>
       <c r="D31">
         <v>108</v>
       </c>
-      <c r="E31" s="27">
+      <c r="E31" s="23">
         <v>0.29166666666666669</v>
       </c>
-      <c r="F31" s="28">
+      <c r="F31" s="24">
         <v>0.33333333333333331</v>
       </c>
-      <c r="G31" s="69" t="s">
+      <c r="G31" s="68" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="18" t="s">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="22">
+      <c r="B32" s="18">
         <v>2</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="18" t="s">
         <v>75</v>
       </c>
       <c r="D32">
         <v>180</v>
       </c>
-      <c r="E32" s="27">
+      <c r="E32" s="23">
         <v>0.6875</v>
       </c>
-      <c r="F32" s="28">
+      <c r="F32" s="24">
         <v>0.72916666666666663</v>
       </c>
-      <c r="G32" s="70"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="18" t="s">
+      <c r="G32" s="69"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B33" s="22">
+      <c r="B33" s="18">
         <v>4</v>
       </c>
-      <c r="C33" s="22" t="s">
+      <c r="C33" s="18" t="s">
         <v>75</v>
       </c>
       <c r="D33">
         <v>180</v>
       </c>
-      <c r="E33" s="27">
+      <c r="E33" s="23">
         <v>0.72916666666666663</v>
       </c>
-      <c r="F33" s="28">
+      <c r="F33" s="24">
         <v>0.91666666666666663</v>
       </c>
-      <c r="G33" s="70"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="18" t="s">
+      <c r="G33" s="69"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B34" s="22">
+      <c r="B34" s="18">
         <v>2</v>
       </c>
-      <c r="C34" s="22" t="s">
+      <c r="C34" s="18" t="s">
         <v>75</v>
       </c>
       <c r="D34">
         <v>180</v>
       </c>
-      <c r="E34" s="27">
+      <c r="E34" s="23">
         <v>0.91666666666666663</v>
       </c>
-      <c r="F34" s="28">
+      <c r="F34" s="24">
         <v>0.95833333333333337</v>
       </c>
-      <c r="G34" s="70"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="17" t="s">
+      <c r="G34" s="69"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B35" s="29">
+      <c r="B35" s="25">
         <v>4</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="25" t="s">
         <v>76</v>
       </c>
       <c r="D35" s="1">
         <v>72</v>
       </c>
-      <c r="E35" s="30">
+      <c r="E35" s="26">
         <v>0</v>
       </c>
-      <c r="F35" s="31">
+      <c r="F35" s="27">
         <v>0.29166666666666669</v>
       </c>
-      <c r="G35" s="70"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="18" t="s">
+      <c r="G35" s="69"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="B36" s="22">
+      <c r="B36" s="18">
         <v>2</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="C36" s="18" t="s">
         <v>76</v>
       </c>
       <c r="D36">
         <v>72</v>
       </c>
-      <c r="E36" s="27">
+      <c r="E36" s="23">
         <v>0.91666666666666663</v>
       </c>
-      <c r="F36" s="32">
+      <c r="F36" s="28">
         <v>0.95833333333333337</v>
       </c>
-      <c r="G36" s="70"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
+      <c r="G36" s="69"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B37" s="26">
+      <c r="B37" s="22">
         <v>4</v>
       </c>
-      <c r="C37" s="26" t="s">
+      <c r="C37" s="22" t="s">
         <v>76</v>
       </c>
       <c r="D37" s="3">
         <v>72</v>
       </c>
-      <c r="E37" s="33">
+      <c r="E37" s="29">
         <v>0.95833333333333337</v>
       </c>
-      <c r="F37" s="34">
+      <c r="F37" s="30">
         <v>1</v>
       </c>
-      <c r="G37" s="71"/>
+      <c r="G37" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2625,410 +2629,410 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E4577B4-9464-4009-9E47-F66B17F055E7}">
   <dimension ref="B2:H32"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="65" t="s">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="64" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="F2" s="65" t="s">
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
+      <c r="F2" s="64" t="s">
         <v>127</v>
       </c>
-      <c r="G2" s="65"/>
-      <c r="H2" s="65"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="16" t="s">
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B3" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="13" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B4" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="F4" s="79">
+      <c r="D4" s="13"/>
+      <c r="F4" s="53">
         <v>0.28472222222222221</v>
       </c>
-      <c r="G4" s="79">
+      <c r="G4" s="53">
         <v>0.28819444444444448</v>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="13">
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B5" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="13">
         <v>8.2999999999999998E-5</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="F5" s="79">
+      <c r="F5" s="53">
         <v>0.28819444444444448</v>
       </c>
-      <c r="G5" s="79">
+      <c r="G5" s="53">
         <v>0.29166666666666669</v>
       </c>
-      <c r="H5" s="16">
+      <c r="H5" s="13">
         <v>0.72</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="16" t="s">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B6" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="13">
         <v>1.3</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="79">
+      <c r="F6" s="53">
         <v>0.29166666666666669</v>
       </c>
-      <c r="G6" s="79">
+      <c r="G6" s="53">
         <v>0.2951388888888889</v>
       </c>
-      <c r="H6" s="16">
+      <c r="H6" s="13">
         <v>0.72499999999999998</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="16" t="s">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B7" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="C7" s="78">
+      <c r="C7" s="52">
         <v>1</v>
       </c>
-      <c r="D7" s="16"/>
-      <c r="F7" s="79">
+      <c r="D7" s="13"/>
+      <c r="F7" s="53">
         <v>0.2951388888888889</v>
       </c>
-      <c r="G7" s="79">
+      <c r="G7" s="53">
         <v>0.32291666666666669</v>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="16" t="s">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B8" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="F8" s="79">
+      <c r="D8" s="13"/>
+      <c r="F8" s="53">
         <v>0.32291666666666669</v>
       </c>
-      <c r="G8" s="79">
+      <c r="G8" s="53">
         <v>0.3263888888888889</v>
       </c>
-      <c r="H8" s="16">
+      <c r="H8" s="13">
         <v>0.65</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B9" s="16" t="s">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B9" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="13">
         <v>2</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="13" t="s">
         <v>102</v>
       </c>
-      <c r="F9" s="79">
+      <c r="F9" s="53">
         <v>0.3263888888888889</v>
       </c>
-      <c r="G9" s="79">
+      <c r="G9" s="53">
         <v>0.3298611111111111</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="13">
         <v>0.74</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F10" s="79">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F10" s="53">
         <v>0.3298611111111111</v>
       </c>
-      <c r="G10" s="79">
+      <c r="G10" s="53">
         <v>0.33333333333333331</v>
       </c>
-      <c r="H10" s="16">
+      <c r="H10" s="13">
         <v>0.08</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F11" s="79">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F11" s="53">
         <v>0.33333333333333331</v>
       </c>
-      <c r="G11" s="79">
+      <c r="G11" s="53">
         <v>0.77083333333333337</v>
       </c>
-      <c r="H11" s="16">
+      <c r="H11" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F12" s="79">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F12" s="53">
         <v>0.77083333333333337</v>
       </c>
-      <c r="G12" s="79">
+      <c r="G12" s="53">
         <v>0.77430555555555547</v>
       </c>
-      <c r="H12" s="16">
+      <c r="H12" s="13">
         <v>0.67</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F13" s="79">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F13" s="53">
         <v>0.77430555555555547</v>
       </c>
-      <c r="G13" s="79">
+      <c r="G13" s="53">
         <v>0.77777777777777779</v>
       </c>
-      <c r="H13" s="16">
+      <c r="H13" s="13">
         <v>0.74</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F14" s="79">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F14" s="53">
         <v>0.77777777777777779</v>
       </c>
-      <c r="G14" s="79">
+      <c r="G14" s="53">
         <v>0.78125</v>
       </c>
-      <c r="H14" s="16">
+      <c r="H14" s="13">
         <v>0.24</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F15" s="79">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F15" s="53">
         <v>0.78125</v>
       </c>
-      <c r="G15" s="79">
+      <c r="G15" s="53">
         <v>0.79166666666666663</v>
       </c>
-      <c r="H15" s="16">
+      <c r="H15" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F16" s="79">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="F16" s="53">
         <v>0.79166666666666663</v>
       </c>
-      <c r="G16" s="79">
+      <c r="G16" s="53">
         <v>0.79513888888888884</v>
       </c>
-      <c r="H16" s="16">
+      <c r="H16" s="13">
         <v>0.4</v>
       </c>
     </row>
-    <row r="17" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F17" s="79">
+    <row r="17" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F17" s="53">
         <v>0.79513888888888884</v>
       </c>
-      <c r="G17" s="79">
+      <c r="G17" s="53">
         <v>0.79861111111111116</v>
       </c>
-      <c r="H17" s="16">
+      <c r="H17" s="13">
         <v>0.09</v>
       </c>
     </row>
-    <row r="18" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F18" s="79">
+    <row r="18" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F18" s="53">
         <v>0.79861111111111116</v>
       </c>
-      <c r="G18" s="79">
+      <c r="G18" s="53">
         <v>0.80902777777777779</v>
       </c>
-      <c r="H18" s="16">
+      <c r="H18" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F19" s="79">
+    <row r="19" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F19" s="53">
         <v>0.80902777777777779</v>
       </c>
-      <c r="G19" s="79">
+      <c r="G19" s="53">
         <v>0.8125</v>
       </c>
-      <c r="H19" s="16">
+      <c r="H19" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F20" s="79">
+    <row r="20" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F20" s="53">
         <v>0.8125</v>
       </c>
-      <c r="G20" s="79">
+      <c r="G20" s="53">
         <v>0.81597222222222221</v>
       </c>
-      <c r="H20" s="16">
+      <c r="H20" s="13">
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="21" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F21" s="79">
+    <row r="21" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F21" s="53">
         <v>0.81597222222222221</v>
       </c>
-      <c r="G21" s="79">
+      <c r="G21" s="53">
         <v>0.81944444444444453</v>
       </c>
-      <c r="H21" s="16">
+      <c r="H21" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F22" s="79">
+    <row r="22" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F22" s="53">
         <v>0.81944444444444453</v>
       </c>
-      <c r="G22" s="79">
+      <c r="G22" s="53">
         <v>0.83333333333333337</v>
       </c>
-      <c r="H22" s="16">
+      <c r="H22" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F23" s="79">
+    <row r="23" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F23" s="53">
         <v>0.83333333333333337</v>
       </c>
-      <c r="G23" s="79">
+      <c r="G23" s="53">
         <v>0.83680555555555547</v>
       </c>
-      <c r="H23" s="16">
+      <c r="H23" s="13">
         <v>0.21</v>
       </c>
     </row>
-    <row r="24" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F24" s="79">
+    <row r="24" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F24" s="53">
         <v>0.83680555555555547</v>
       </c>
-      <c r="G24" s="79">
+      <c r="G24" s="53">
         <v>0.86458333333333337</v>
       </c>
-      <c r="H24" s="16">
+      <c r="H24" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F25" s="79">
+    <row r="25" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F25" s="53">
         <v>0.86458333333333337</v>
       </c>
-      <c r="G25" s="79">
+      <c r="G25" s="53">
         <v>0.86805555555555547</v>
       </c>
-      <c r="H25" s="16">
+      <c r="H25" s="13">
         <v>0.21</v>
       </c>
     </row>
-    <row r="26" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F26" s="79">
+    <row r="26" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F26" s="53">
         <v>0.86805555555555547</v>
       </c>
-      <c r="G26" s="79">
+      <c r="G26" s="53">
         <v>0.875</v>
       </c>
-      <c r="H26" s="16">
+      <c r="H26" s="13">
         <v>0.08</v>
       </c>
     </row>
-    <row r="27" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F27" s="79">
+    <row r="27" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F27" s="53">
         <v>0.875</v>
       </c>
-      <c r="G27" s="79">
+      <c r="G27" s="53">
         <v>0.87847222222222221</v>
       </c>
-      <c r="H27" s="16">
+      <c r="H27" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F28" s="79">
+    <row r="28" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F28" s="53">
         <v>0.87847222222222221</v>
       </c>
-      <c r="G28" s="79">
+      <c r="G28" s="53">
         <v>0.88194444444444453</v>
       </c>
-      <c r="H28" s="16">
+      <c r="H28" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F29" s="79">
+    <row r="29" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F29" s="53">
         <v>0.88194444444444453</v>
       </c>
-      <c r="G29" s="79">
+      <c r="G29" s="53">
         <v>0.9375</v>
       </c>
-      <c r="H29" s="16">
+      <c r="H29" s="13">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F30" s="79">
+    <row r="30" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F30" s="53">
         <v>0.9375</v>
       </c>
-      <c r="G30" s="79">
+      <c r="G30" s="53">
         <v>0.94097222222222221</v>
       </c>
-      <c r="H30" s="16">
+      <c r="H30" s="13">
         <v>0.63</v>
       </c>
     </row>
-    <row r="31" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F31" s="79">
+    <row r="31" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F31" s="53">
         <v>0.94097222222222221</v>
       </c>
-      <c r="G31" s="79">
+      <c r="G31" s="53">
         <v>0.94791666666666663</v>
       </c>
-      <c r="H31" s="16">
+      <c r="H31" s="13">
         <v>0.73</v>
       </c>
     </row>
-    <row r="32" spans="6:8" x14ac:dyDescent="0.25">
-      <c r="F32" s="79">
+    <row r="32" spans="6:8" x14ac:dyDescent="0.35">
+      <c r="F32" s="53">
         <v>0.94791666666666663</v>
       </c>
-      <c r="G32" s="80">
+      <c r="G32" s="54">
         <v>1</v>
       </c>
-      <c r="H32" s="16">
+      <c r="H32" s="13">
         <v>0</v>
       </c>
     </row>
@@ -3044,14 +3048,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB2FBFAB-6257-4B0F-A03C-5C54BAFB6B00}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>123</v>
       </c>
@@ -3062,7 +3066,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>120</v>
       </c>
@@ -3070,7 +3074,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>107</v>
       </c>
@@ -3081,7 +3085,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>108</v>
       </c>
@@ -3092,7 +3096,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>109</v>
       </c>
@@ -3103,7 +3107,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>110</v>
       </c>
@@ -3114,7 +3118,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>113</v>
       </c>
@@ -3125,7 +3129,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>112</v>
       </c>

</xml_diff>